<commit_message>
Lab 3 MatStat full completed
</commit_message>
<xml_diff>
--- a/3сем/ТВиМС/Lab3/ЛР3 Критерии значимости.xlsx
+++ b/3сем/ТВиМС/Lab3/ЛР3 Критерии значимости.xlsx
@@ -380,15 +380,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>205740</xdr:colOff>
+      <xdr:colOff>205741</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:rowOff>99061</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>5359</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>110397</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>556261</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>118939</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -405,8 +405,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7094220" y="99060"/>
-          <a:ext cx="2847619" cy="742857"/>
+          <a:off x="7094221" y="99061"/>
+          <a:ext cx="2179320" cy="568518"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -417,16 +417,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>589433</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>26444</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>398933</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>92928</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -443,8 +443,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3421380" y="1333500"/>
-          <a:ext cx="8933333" cy="1809524"/>
+          <a:off x="4617720" y="1013460"/>
+          <a:ext cx="6327293" cy="1281648"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -455,16 +455,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>7620</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>327660</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>19</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -473,8 +473,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3581400" y="3307080"/>
-          <a:ext cx="8374380" cy="815340"/>
+          <a:off x="4168140" y="2324100"/>
+          <a:ext cx="7726680" cy="746760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -561,16 +561,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>449580</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>22860</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>40582</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>391370</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>157892</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>40850</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>165511</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -587,14 +587,148 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3680460" y="4244340"/>
-          <a:ext cx="8476190" cy="1780952"/>
+          <a:off x="4472940" y="3157162"/>
+          <a:ext cx="6723590" cy="1412709"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>388620</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4229100" y="4709160"/>
+          <a:ext cx="7764780" cy="784860"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>Поскольку</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>t</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>расч </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>&gt; t</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>табл, то делаем вывод</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>: </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>на уровне значимости 0,05 можно утверждать, что </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>H0</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t> противоречит экспериментальным данным, т.е. различия между результатами измерений у мужчин и женщин следует признать значительными.</a:t>
+          </a:r>
+          <a:endParaRPr lang="ru-RU" sz="1400">
+            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -604,16 +738,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>487680</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>20480</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>137065</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>256700</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>83725</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -630,7 +764,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8519160" y="1211580"/>
+          <a:off x="11193780" y="236220"/>
           <a:ext cx="3800000" cy="761905"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -642,16 +776,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>320040</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>218643</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>26534</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>119583</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>57014</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -668,7 +802,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8450580" y="2065020"/>
+          <a:off x="7132320" y="1173480"/>
           <a:ext cx="3457143" cy="1085714"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -680,16 +814,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>472440</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>110373</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>102753</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>29394</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>127279</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>67494</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>112039</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -706,7 +840,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8503920" y="3417453"/>
+          <a:off x="7322820" y="2304933"/>
           <a:ext cx="5652954" cy="1853326"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -719,15 +853,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>571499</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>426721</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>3560</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>98146</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -744,8 +878,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1" y="4061460"/>
-          <a:ext cx="8458200" cy="2000000"/>
+          <a:off x="571499" y="4061460"/>
+          <a:ext cx="6537961" cy="1545946"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -757,15 +891,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>68580</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>251460</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -774,7 +908,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="68580" y="6286500"/>
+          <a:off x="160020" y="5699760"/>
           <a:ext cx="8214360" cy="944880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -921,16 +1055,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>647700</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>426582</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>137112</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>68442</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>99012</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -947,7 +1081,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="647700" y="7277100"/>
+          <a:off x="899160" y="6690360"/>
           <a:ext cx="1104762" cy="380952"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -960,15 +1094,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>491197</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>22817</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>72097</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>121877</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -985,7 +1119,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="83820" y="7749540"/>
+          <a:off x="274320" y="7117080"/>
           <a:ext cx="2342857" cy="342857"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -998,15 +1132,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>175260</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>51298</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>47581</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>516118</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>131401</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1023,7 +1157,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2720340" y="7764780"/>
+          <a:off x="2575560" y="7117080"/>
           <a:ext cx="1095238" cy="352381"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1036,15 +1170,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:colOff>525780</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>535090</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>116156</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>420790</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>39956</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1061,7 +1195,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8671560" y="5966460"/>
+          <a:off x="9166860" y="4244340"/>
           <a:ext cx="1723810" cy="390476"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1073,16 +1207,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>541020</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>7534</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>165679</xdr:rowOff>
+      <xdr:colOff>419014</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>97099</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1099,7 +1233,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10401300" y="5958840"/>
+          <a:off x="10812780" y="4244340"/>
           <a:ext cx="685714" cy="447619"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1112,15 +1246,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>586740</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:colOff>106680</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>129540</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1129,7 +1263,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8618220" y="6492240"/>
+          <a:off x="8138160" y="4815840"/>
           <a:ext cx="6149340" cy="609600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1179,15 +1313,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>502920</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>17077</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>104729</xdr:rowOff>
+      <xdr:colOff>436177</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>173309</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1204,7 +1338,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8724900" y="7437120"/>
+          <a:off x="9144000" y="5494020"/>
           <a:ext cx="542857" cy="371429"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1217,15 +1351,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>449580</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>36115</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>158064</xdr:rowOff>
+      <xdr:colOff>478075</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>36144</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1242,7 +1376,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9258300" y="7452360"/>
+          <a:off x="9700260" y="5501640"/>
           <a:ext cx="638095" cy="409524"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1254,16 +1388,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>121920</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>24</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>472440</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1272,7 +1406,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="8694420" y="8008620"/>
+          <a:off x="8450580" y="5958840"/>
           <a:ext cx="6149340" cy="1074420"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1326,7 +1460,21 @@
               <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
               <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
             </a:rPr>
-            <a:t>не противоречит экспериментальным данным, т. е. нет оснований утверждать, что при использовании сухой смеси время литья значимо уменьшится.</a:t>
+            <a:t>не противоречит экспериментальным данным, т. е. нет оснований утверждать, что происходит</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400" baseline="0">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t> систематическое изменение стока из года в год</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="ru-RU" sz="1400">
+              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+            </a:rPr>
+            <a:t>.</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>